<commit_message>
Update approved budget workbook
</commit_message>
<xml_diff>
--- a/data/11505/各系核定經費及各類經費明細與系所代碼.xlsx
+++ b/data/11505/各系核定經費及各類經費明細與系所代碼.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\IR大數據分析組\IR-躍升相關\經費收支明細\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\projects\BudgetDashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{814583A1-E610-4FEB-8DAC-A99CC782E202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09949E15-5FC5-4089-9F9F-F7B5424DA8BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{DEB7F6D8-750E-40F3-B511-66BA571B0662}"/>
   </bookViews>
@@ -518,15 +518,110 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>以業務費</t>
+    <t>UP04</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>會計資訊系</t>
+    </r>
+  </si>
+  <si>
+    <t>UT01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>智慧商務系</t>
+    </r>
+  </si>
+  <si>
+    <t>UQ01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>造船及海洋工程系</t>
+    </r>
+  </si>
+  <si>
+    <t>UC11</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>國際企業系</t>
+    </r>
+  </si>
+  <si>
+    <t>UV01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>商務資訊應用系</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>海洋商務學院</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1.(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>業務費</t>
     </r>
     <r>
       <rPr>
@@ -535,17 +630,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>-173,800</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>元與工管系交換無形資產</t>
+      <t>+103,142)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>與風管系、國企系合辦國際研討會，並統一由財管系報支，兩系授權業務費共計</t>
     </r>
     <r>
       <rPr>
@@ -554,158 +649,205 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>173,800</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>元</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>UP04</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>會計資訊系</t>
-    </r>
-  </si>
-  <si>
-    <t>UT01</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>智慧商務系</t>
-    </r>
-  </si>
-  <si>
-    <t>UQ01</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>造船及海洋工程系</t>
-    </r>
-  </si>
-  <si>
-    <t>UC11</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>國際企業系</t>
-    </r>
-  </si>
-  <si>
-    <t>UV01</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>商務資訊應用系</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>海洋商務學院</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>1.(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>業務費</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
+      <t>103,142</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>元。</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UP03</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>財務管理系</t>
+    </r>
+  </si>
+  <si>
+    <t>UT03</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>財政稅務系</t>
+    </r>
+  </si>
+  <si>
+    <t>UO01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>航運管理系</t>
+    </r>
+  </si>
+  <si>
+    <t>UR01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>航運技術系</t>
+    </r>
+  </si>
+  <si>
+    <t>UQ04</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>海洋環境工程系</t>
+    </r>
+  </si>
+  <si>
+    <t>UR03</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>海事資訊科技系</t>
+    </r>
+  </si>
+  <si>
+    <t>UO04</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>海洋休閒管理系</t>
+    </r>
+  </si>
+  <si>
+    <t>US04</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>海洋生物技術系</t>
+    </r>
+  </si>
+  <si>
+    <t>UP02</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>風險管理與保險系</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>以國外旅費</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>+103,142)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>與風管系、國企系合辦國際研討會，並統一由財管系報支，兩系授權業務費共計</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
+      <t>74,000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>元與國企系交換業務費</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>103,142</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
+      <t>74,000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
         <rFont val="標楷體"/>
         <family val="4"/>
         <charset val="136"/>
@@ -715,147 +857,147 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>UP03</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>財務管理系</t>
-    </r>
-  </si>
-  <si>
-    <t>UT03</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>財政稅務系</t>
-    </r>
-  </si>
-  <si>
-    <t>UO01</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>航運管理系</t>
-    </r>
-  </si>
-  <si>
-    <t>UR01</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>航運技術系</t>
-    </r>
-  </si>
-  <si>
-    <t>UQ04</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>海洋環境工程系</t>
-    </r>
-  </si>
-  <si>
-    <t>UR03</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>海事資訊科技系</t>
-    </r>
-  </si>
-  <si>
-    <t>UO04</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>海洋休閒管理系</t>
-    </r>
-  </si>
-  <si>
-    <t>US04</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>海洋生物技術系</t>
-    </r>
-  </si>
-  <si>
-    <t>UP02</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>風險管理與保險系</t>
+    <t>UN03</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>科技法律研究所</t>
+    </r>
+  </si>
+  <si>
+    <t>UP01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>金融系</t>
+    </r>
+  </si>
+  <si>
+    <t>UC45</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>金融資訊系</t>
+    </r>
+  </si>
+  <si>
+    <t>UO03</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>供應鏈管理系</t>
+    </r>
+  </si>
+  <si>
+    <t>UN04</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>行銷與流通管理系</t>
+    </r>
+  </si>
+  <si>
+    <t>UM74</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>企業管理系</t>
+    </r>
+  </si>
+  <si>
+    <t>UB03</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>半導體工程系</t>
+    </r>
+  </si>
+  <si>
+    <t>US02</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>水產食品科學系</t>
+    </r>
+  </si>
+  <si>
+    <t>UE16</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>化學工程與材料工程系</t>
     </r>
   </si>
   <si>
@@ -865,205 +1007,275 @@
     <r>
       <rPr>
         <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>以國外旅費</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>以無形資產</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>74,000</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>元與國企系交換業務費</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
+      <t>-173,800</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>元與會資系交換業務費</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>74,000</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>元。</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>UN03</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>科技法律研究所</t>
-    </r>
-  </si>
-  <si>
-    <t>UP01</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>金融系</t>
-    </r>
-  </si>
-  <si>
-    <t>UC45</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>金融資訊系</t>
-    </r>
-  </si>
-  <si>
-    <t>UO03</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>供應鏈管理系</t>
-    </r>
-  </si>
-  <si>
-    <t>UN04</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>行銷與流通管理系</t>
-    </r>
-  </si>
-  <si>
-    <t>UM74</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>企業管理系</t>
-    </r>
-  </si>
-  <si>
-    <t>UB03</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>半導體工程系</t>
-    </r>
-  </si>
-  <si>
-    <t>US02</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>水產食品科學系</t>
-    </r>
-  </si>
-  <si>
-    <t>UE16</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>化學工程與材料工程系</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>1.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>以無形資產</t>
+      <t>173,800</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UE72</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>工業工程與管理系</t>
+    </r>
+  </si>
+  <si>
+    <t>工學院</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UF08</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>工業設計系</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>創新設計學院</t>
+    </r>
+  </si>
+  <si>
+    <t>UE23</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>土木工程系</t>
+    </r>
+  </si>
+  <si>
+    <t>UH53</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>人力資源發展系</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>設備費</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>無形資產</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>大陸地區旅費</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>國外旅費</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>業務費</t>
+    </r>
+  </si>
+  <si>
+    <t>業務費餘額</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>實支率</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>實支數</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>動支率</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>動支數</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>調整說明</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>兩期合計</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>第二期</t>
     </r>
     <r>
       <rPr>
@@ -1072,17 +1284,30 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>-173,800</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>元與會資系交換業務費</t>
+      <t>(115TSD00-8)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>撥付</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>第一期</t>
     </r>
     <r>
       <rPr>
@@ -1091,242 +1316,51 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>173,800</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>元</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>UE72</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>工業工程與管理系</t>
-    </r>
-  </si>
-  <si>
-    <t>工學院</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>UF08</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>工業設計系</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>創新設計學院</t>
-    </r>
-  </si>
-  <si>
-    <t>UE23</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>土木工程系</t>
-    </r>
-  </si>
-  <si>
-    <t>UH53</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>人力資源發展系</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>設備費</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>無形資產</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>大陸地區旅費</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>國外旅費</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>業務費</t>
-    </r>
-  </si>
-  <si>
-    <t>業務費餘額</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>實支率</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>實支數</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>動支率</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>動支數</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>調整說明</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>兩期合計</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>第二期</t>
+      <t>(114TSD00-15)</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>帳號</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>系所</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>學院</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>115.06</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>專簽奉准，設備費</t>
     </r>
     <r>
       <rPr>
@@ -1335,30 +1369,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>(115TSD00-8)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>撥付</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>第一期</t>
+      <t>140</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>萬調整為設備費</t>
     </r>
     <r>
       <rPr>
@@ -1367,51 +1388,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>(114TSD00-15)</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>帳號</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>系所</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>學院</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>115.06</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>專簽奉准，設備費</t>
+      <t>92</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>萬與無形資產</t>
     </r>
     <r>
       <rPr>
@@ -1420,17 +1407,33 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>140</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>萬調整為設備費</t>
+      <t>48</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>萬。</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -1439,17 +1442,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>92</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>萬與無形資產</t>
+      <t>6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>月國企系授權設備費$</t>
     </r>
     <r>
       <rPr>
@@ -1458,33 +1461,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>48</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>萬。</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>.</t>
+      <t>26,415</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>與金資系合購設備</t>
     </r>
     <r>
       <rPr>
@@ -1493,17 +1480,81 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>6</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>月國企系授權設備費$</t>
+      <t xml:space="preserve">
+2.6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>月授權328元給國企系</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>7月以國外旅費-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>70,000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>元與電機系交換設備費</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>70,000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>7月以設備費-70,000元與供應鏈系交換國外旅費70,000元</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>1.商資系用國外旅費</t>
     </r>
     <r>
       <rPr>
@@ -1512,17 +1563,33 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>26,415</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>與金資系合購設備</t>
+      <t>$16,995</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>與風管系交換業務費</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>1.(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>設備費</t>
     </r>
     <r>
       <rPr>
@@ -1531,81 +1598,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve">
-2.6</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>月授權328元給國企系</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>7月以國外旅費-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>70,000</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>元與電機系交換設備費</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>70,000</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>元</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>7月以設備費-70,000元與供應鏈系交換國外旅費70,000元</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>1.商資系用國外旅費</t>
+      <t>+5723)114</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>年國企系設備費超支</t>
     </r>
     <r>
       <rPr>
@@ -1614,33 +1617,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>$16,995</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>與風管系交換業務費</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>1.(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>設備費</t>
+      <t>$5723</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>，向風管系借，</t>
     </r>
     <r>
       <rPr>
@@ -1649,17 +1636,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>+5723)114</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>年國企系設備費超支</t>
+      <t>115</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>年國企系還</t>
     </r>
     <r>
       <rPr>
@@ -1668,17 +1655,18 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>$5723</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>，向風管系借，</t>
+      <t>$5723
+2.(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>業務費</t>
     </r>
     <r>
       <rPr>
@@ -1687,17 +1675,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>115</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>年國企系還</t>
+      <t>-51,571)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>與財管系合辦國際研討會，並統一由財管系報支，授權業務費</t>
     </r>
     <r>
       <rPr>
@@ -1706,18 +1694,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>$5723
-2.(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>業務費</t>
+      <t>51,571</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>給財管系。</t>
     </r>
     <r>
       <rPr>
@@ -1726,17 +1713,18 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>-51,571)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>與財管系合辦國際研討會，並統一由財管系報支，授權業務費</t>
+      <t xml:space="preserve">
+3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>商資系用國外旅費</t>
     </r>
     <r>
       <rPr>
@@ -1745,71 +1733,66 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>51,571</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>給財管系。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
+      <t>$16,995</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>與風管系交換業務費</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>1.(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>設備費</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve">
-3.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>商資系用國外旅費</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
+      <t>-5723)114</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>年設備費超支</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>$16,995</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>與風管系交換業務費</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>1.(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>設備費</t>
+      <t>$5723</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>，向風管系借，</t>
     </r>
     <r>
       <rPr>
@@ -1817,16 +1800,16 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>-5723)114</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>年設備費超支</t>
+      <t>115</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>年還</t>
     </r>
     <r>
       <rPr>
@@ -1834,16 +1817,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>$5723</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>，向風管系借，</t>
+      <t>$5723
+2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>以業務費</t>
     </r>
     <r>
       <rPr>
@@ -1851,16 +1835,16 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>115</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>年還</t>
+      <t>74,000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>元與科法所交換國外旅費</t>
     </r>
     <r>
       <rPr>
@@ -1868,17 +1852,25 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>$5723
-2.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>以業務費</t>
+      <t>74,000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>元。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="4"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
     </r>
     <r>
       <rPr>
@@ -1886,16 +1878,16 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>74,000</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>元與科法所交換國外旅費</t>
+      <t>3.(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>業務費</t>
     </r>
     <r>
       <rPr>
@@ -1903,17 +1895,16 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>74,000</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">元。
-</t>
+      <t>-51,571)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>與財管系合辦國際研討會，並統一由財管系報支，授權業務費</t>
     </r>
     <r>
       <rPr>
@@ -1921,16 +1912,16 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>3.(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>業務費</t>
+      <t>51,571</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>給財管系。</t>
     </r>
     <r>
       <rPr>
@@ -1938,16 +1929,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>-51,571)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>與財管系合辦國際研討會，並統一由財管系報支，授權業務費</t>
+      <t xml:space="preserve">
+4.6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>月份與金資系合購設備，授權設備費</t>
     </r>
     <r>
       <rPr>
@@ -1955,16 +1947,16 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>51,571</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>給財管系。</t>
+      <t>$26,415</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>給金資系。</t>
     </r>
     <r>
       <rPr>
@@ -1973,7 +1965,7 @@
         <family val="1"/>
       </rPr>
       <t xml:space="preserve">
-4.6</t>
+5.6</t>
     </r>
     <r>
       <rPr>
@@ -1982,7 +1974,7 @@
         <family val="1"/>
         <charset val="136"/>
       </rPr>
-      <t>月份與金資系合購設備，授權設備費</t>
+      <t>月</t>
     </r>
     <r>
       <rPr>
@@ -1990,7 +1982,7 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>$26,415</t>
+      <t>30</t>
     </r>
     <r>
       <rPr>
@@ -1999,7 +1991,7 @@
         <family val="1"/>
         <charset val="136"/>
       </rPr>
-      <t>給金資系。</t>
+      <t>日，從金資系授權</t>
     </r>
     <r>
       <rPr>
@@ -2007,8 +1999,7 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve">
-5.6</t>
+      <t>$328</t>
     </r>
     <r>
       <rPr>
@@ -2017,7 +2008,7 @@
         <family val="1"/>
         <charset val="136"/>
       </rPr>
-      <t>月</t>
+      <t>業務費到國企系</t>
     </r>
     <r>
       <rPr>
@@ -2025,7 +2016,8 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>30</t>
+      <t xml:space="preserve">
+6.</t>
     </r>
     <r>
       <rPr>
@@ -2034,7 +2026,7 @@
         <family val="1"/>
         <charset val="136"/>
       </rPr>
-      <t>日，從金資系授權</t>
+      <t>國企系以設備費</t>
     </r>
     <r>
       <rPr>
@@ -2042,7 +2034,7 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>$328</t>
+      <t>6000</t>
     </r>
     <r>
       <rPr>
@@ -2051,7 +2043,105 @@
         <family val="1"/>
         <charset val="136"/>
       </rPr>
-      <t>業務費到國企系</t>
+      <t>與會資系交換業務費</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>6000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="標楷體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="4"/>
+      </rPr>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>以業務費</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>-173,800</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>元與工管系交換無形資產</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>173,800</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>元</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">
+2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>國企系以設備費6000與會資系交換業務費6000元</t>
     </r>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -2064,7 +2154,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="176" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2156,6 +2246,11 @@
       <family val="1"/>
       <charset val="136"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="4"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -2642,7 +2737,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2816,6 +2911,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3210,86 +3308,86 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="63" t="s">
-        <v>126</v>
-      </c>
-      <c r="B1" s="65" t="s">
+      <c r="A1" s="64" t="s">
         <v>125</v>
       </c>
-      <c r="C1" s="67" t="s">
+      <c r="B1" s="66" t="s">
         <v>124</v>
       </c>
-      <c r="D1" s="69" t="s">
+      <c r="C1" s="68" t="s">
         <v>123</v>
       </c>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72" t="s">
+      <c r="D1" s="70" t="s">
         <v>122</v>
       </c>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="74"/>
-      <c r="O1" s="75" t="s">
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="73" t="s">
         <v>121</v>
       </c>
-      <c r="P1" s="58" t="s">
+      <c r="K1" s="74"/>
+      <c r="L1" s="74"/>
+      <c r="M1" s="74"/>
+      <c r="N1" s="75"/>
+      <c r="O1" s="76" t="s">
         <v>120</v>
+      </c>
+      <c r="P1" s="59" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="64"/>
-      <c r="B2" s="66"/>
-      <c r="C2" s="68"/>
+      <c r="A2" s="65"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="69"/>
       <c r="D2" s="55" t="s">
+        <v>113</v>
+      </c>
+      <c r="E2" s="54" t="s">
+        <v>118</v>
+      </c>
+      <c r="F2" s="54" t="s">
+        <v>117</v>
+      </c>
+      <c r="G2" s="54" t="s">
+        <v>116</v>
+      </c>
+      <c r="H2" s="54" t="s">
+        <v>115</v>
+      </c>
+      <c r="I2" s="53" t="s">
         <v>114</v>
       </c>
-      <c r="E2" s="54" t="s">
-        <v>119</v>
-      </c>
-      <c r="F2" s="54" t="s">
-        <v>118</v>
-      </c>
-      <c r="G2" s="54" t="s">
-        <v>117</v>
-      </c>
-      <c r="H2" s="54" t="s">
-        <v>116</v>
-      </c>
-      <c r="I2" s="53" t="s">
-        <v>115</v>
-      </c>
       <c r="J2" s="52" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K2" s="51" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L2" s="51" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="M2" s="51" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N2" s="50" t="s">
-        <v>110</v>
-      </c>
-      <c r="O2" s="76"/>
-      <c r="P2" s="59"/>
+        <v>109</v>
+      </c>
+      <c r="O2" s="77"/>
+      <c r="P2" s="60"/>
     </row>
     <row r="3" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="49" t="s">
         <v>44</v>
       </c>
       <c r="B3" s="48" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D3" s="46">
         <v>400000</v>
@@ -3338,10 +3436,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D4" s="24">
         <v>400000</v>
@@ -3387,13 +3485,13 @@
     </row>
     <row r="5" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D5" s="24">
         <v>400000</v>
@@ -3439,13 +3537,13 @@
     </row>
     <row r="6" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="36" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D6" s="24">
         <v>400000</v>
@@ -3486,7 +3584,7 @@
         <v>2000000</v>
       </c>
       <c r="P6" s="33" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3494,10 +3592,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D7" s="24">
         <v>400000</v>
@@ -3542,10 +3640,10 @@
         <v>23</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D8" s="24">
         <v>400000</v>
@@ -3590,10 +3688,10 @@
         <v>33</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D9" s="24">
         <v>400000</v>
@@ -3642,10 +3740,10 @@
         <v>44</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C10" s="25" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D10" s="24">
         <v>400000</v>
@@ -3694,10 +3792,10 @@
         <v>44</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D11" s="24">
         <v>400000</v>
@@ -3743,13 +3841,13 @@
     </row>
     <row r="12" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D12" s="24">
         <v>400000</v>
@@ -3794,7 +3892,7 @@
         <v>2000000</v>
       </c>
       <c r="P12" s="57" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="33" x14ac:dyDescent="0.25">
@@ -3802,10 +3900,10 @@
         <v>6</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D13" s="24">
         <v>400000</v>
@@ -3850,7 +3948,7 @@
         <v>2026087</v>
       </c>
       <c r="P13" s="33" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3858,10 +3956,10 @@
         <v>44</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D14" s="24">
         <v>400000</v>
@@ -3906,10 +4004,10 @@
         <v>44</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D15" s="24">
         <v>400000</v>
@@ -3950,7 +4048,7 @@
         <v>2000000</v>
       </c>
       <c r="P15" s="34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="82.5" x14ac:dyDescent="0.25">
@@ -3958,10 +4056,10 @@
         <v>44</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D16" s="24">
         <v>400000</v>
@@ -4003,7 +4101,7 @@
         <v>1954152</v>
       </c>
       <c r="P16" s="33" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -4011,10 +4109,10 @@
         <v>23</v>
       </c>
       <c r="B17" s="26" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D17" s="24">
         <v>400000</v>
@@ -4056,13 +4154,13 @@
     </row>
     <row r="18" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D18" s="24">
         <v>400000</v>
@@ -4111,10 +4209,10 @@
         <v>26</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D19" s="24">
         <v>400000</v>
@@ -4163,10 +4261,10 @@
         <v>23</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D20" s="24">
         <v>400000</v>
@@ -4211,10 +4309,10 @@
         <v>26</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D21" s="24">
         <v>400000</v>
@@ -4260,13 +4358,13 @@
     </row>
     <row r="22" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D22" s="24">
         <v>400000</v>
@@ -4315,10 +4413,10 @@
         <v>6</v>
       </c>
       <c r="B23" s="26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D23" s="24">
         <v>400000</v>
@@ -4367,10 +4465,10 @@
         <v>44</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D24" s="24">
         <v>400000</v>
@@ -4413,18 +4511,18 @@
         <v>2103142</v>
       </c>
       <c r="P24" s="33" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D25" s="24">
         <v>400000</v>
@@ -4469,18 +4567,18 @@
         <v>2000000</v>
       </c>
       <c r="P25" s="56" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="99" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" ht="115.5" x14ac:dyDescent="0.25">
       <c r="A26" s="27" t="s">
         <v>44</v>
       </c>
       <c r="B26" s="26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C26" s="25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D26" s="24">
         <v>400000</v>
@@ -4504,8 +4602,8 @@
         <v>319171</v>
       </c>
       <c r="J26" s="32">
-        <f>126000-74000+328</f>
-        <v>52328</v>
+        <f>126000-74000+328+6000</f>
+        <v>58328</v>
       </c>
       <c r="K26" s="31">
         <f>74000+74000</f>
@@ -4518,15 +4616,15 @@
         <v>700000</v>
       </c>
       <c r="N26" s="30">
-        <f>700000-5723-26415</f>
-        <v>667862</v>
+        <f>700000-5723-26415-6000</f>
+        <v>661862</v>
       </c>
       <c r="O26" s="8">
         <f t="shared" si="3"/>
         <v>1916619</v>
       </c>
       <c r="P26" s="29" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -4534,10 +4632,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D27" s="24">
         <v>400000</v>
@@ -4586,10 +4684,10 @@
         <v>6</v>
       </c>
       <c r="B28" s="26" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C28" s="25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D28" s="24">
         <v>400000</v>
@@ -4638,10 +4736,10 @@
         <v>6</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C29" s="25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D29" s="24">
         <v>400000</v>
@@ -4664,9 +4762,9 @@
         <f t="shared" si="5"/>
         <v>383294</v>
       </c>
-      <c r="J29" s="22">
-        <f>200000-173800</f>
-        <v>26200</v>
+      <c r="J29" s="32">
+        <f>200000-173800-6000</f>
+        <v>20200</v>
       </c>
       <c r="K29" s="21">
         <v>0</v>
@@ -4678,15 +4776,16 @@
         <f>1020000+173800</f>
         <v>1193800</v>
       </c>
-      <c r="N29" s="20">
-        <v>380000</v>
+      <c r="N29" s="30">
+        <f>380000+6000</f>
+        <v>386000</v>
       </c>
       <c r="O29" s="8">
         <f t="shared" si="3"/>
         <v>2000000</v>
       </c>
-      <c r="P29" s="56" t="s">
-        <v>49</v>
+      <c r="P29" s="58" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="30" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -5086,7 +5185,7 @@
         <v>2000000</v>
       </c>
       <c r="P37" s="57" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="38" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -5230,17 +5329,17 @@
         <v>0</v>
       </c>
       <c r="M40" s="31">
-        <v>48000</v>
+        <v>480000</v>
       </c>
       <c r="N40" s="30">
-        <v>92000</v>
+        <v>920000</v>
       </c>
       <c r="O40" s="8">
         <f t="shared" si="3"/>
-        <v>740000</v>
+        <v>2000000</v>
       </c>
       <c r="P40" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="41" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -5689,11 +5788,11 @@
       <c r="P49" s="7"/>
     </row>
     <row r="50" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B50" s="61"/>
-      <c r="C50" s="62"/>
+      <c r="A50" s="61" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" s="62"/>
+      <c r="C50" s="63"/>
       <c r="D50" s="5">
         <f>SUM(D3:D49)</f>
         <v>18400000</v>
@@ -5732,22 +5831,22 @@
       </c>
       <c r="M50" s="5">
         <f t="shared" si="6"/>
-        <v>7374500</v>
+        <v>7806500</v>
       </c>
       <c r="N50" s="4">
         <f t="shared" si="6"/>
-        <v>57680650</v>
+        <v>58508650</v>
       </c>
       <c r="O50" s="3">
         <f t="shared" si="6"/>
-        <v>92740000</v>
+        <v>94000000</v>
       </c>
       <c r="P50" s="2"/>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="N51" s="1">
         <f>I50+J50+K50+L50+M50+N50</f>
-        <v>91217912</v>
+        <v>92477912</v>
       </c>
     </row>
   </sheetData>

</xml_diff>